<commit_message>
add option in base and modify infos in excel
</commit_message>
<xml_diff>
--- a/TestData/Classeur1.xlsx
+++ b/TestData/Classeur1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mourad\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09D2A401-C855-4F30-B726-793ECF16C163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C86953-5D0D-4D6E-94B1-F46D4429BD61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{5FC3486C-B765-4766-AEA2-A396004EA852}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8964" xr2:uid="{5FC3486C-B765-4766-AEA2-A396004EA852}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>username</t>
   </si>
@@ -62,15 +62,6 @@
     <t>secret_sauce</t>
   </si>
   <si>
-    <t>problem_user</t>
-  </si>
-  <si>
-    <t>wronguser</t>
-  </si>
-  <si>
-    <t>wrongpass</t>
-  </si>
-  <si>
     <t>hamid</t>
   </si>
   <si>
@@ -78,9 +69,6 @@
   </si>
   <si>
     <t>true</t>
-  </si>
-  <si>
-    <t>false</t>
   </si>
   <si>
     <t>performance_glitch_user</t>
@@ -462,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7551AD3-F191-49BB-AC7E-805214165F83}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -493,76 +481,36 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E2">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E3">
-        <v>10000</v>
+        <v>21000</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4">
-        <v>10000</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5">
-        <v>10000</v>
-      </c>
-      <c r="F5" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add wrong_user in excel
</commit_message>
<xml_diff>
--- a/TestData/Classeur1.xlsx
+++ b/TestData/Classeur1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mourad\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C86953-5D0D-4D6E-94B1-F46D4429BD61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FBEF89-E9CC-408A-86C4-B35AFDFD1889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8964" xr2:uid="{5FC3486C-B765-4766-AEA2-A396004EA852}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>username</t>
   </si>
@@ -72,6 +72,21 @@
   </si>
   <si>
     <t>performance_glitch_user</t>
+  </si>
+  <si>
+    <t>wrong_user</t>
+  </si>
+  <si>
+    <t>wrongpass</t>
+  </si>
+  <si>
+    <t>salim</t>
+  </si>
+  <si>
+    <t>zaza</t>
+  </si>
+  <si>
+    <t>false</t>
   </si>
 </sst>
 </file>
@@ -450,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7551AD3-F191-49BB-AC7E-805214165F83}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -513,6 +528,26 @@
         <v>10</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4">
+        <v>20000</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
modify wait in the login and test fail with test pass
</commit_message>
<xml_diff>
--- a/TestData/Classeur1.xlsx
+++ b/TestData/Classeur1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mourad\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FBEF89-E9CC-408A-86C4-B35AFDFD1889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C9A5795-C881-479D-AF6A-676D3A78BDB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8964" xr2:uid="{5FC3486C-B765-4766-AEA2-A396004EA852}"/>
   </bookViews>
@@ -74,9 +74,6 @@
     <t>performance_glitch_user</t>
   </si>
   <si>
-    <t>wrong_user</t>
-  </si>
-  <si>
     <t>wrongpass</t>
   </si>
   <si>
@@ -87,6 +84,9 @@
   </si>
   <si>
     <t>false</t>
+  </si>
+  <si>
+    <t>user_ghalat</t>
   </si>
 </sst>
 </file>
@@ -530,22 +530,22 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
       <c r="E4">
         <v>20000</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>